<commit_message>
Weekly GA4 tables update 2026-09-21 (through week ending 2026-09-20)
</commit_message>
<xml_diff>
--- a/exports/Seeed周度三表_W23-W36_2026-09-20.xlsx
+++ b/exports/Seeed周度三表_W23-W36_2026-09-20.xlsx
@@ -515,19 +515,19 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>327</v>
+        <v>896</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>417</v>
+        <v>1108</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>9.109999999999999</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-53.8</v>
+        <v>22.8</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -536,7 +536,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>应急响应 (+0.0%)</t>
+          <t>应急响应 (+200.0%)</t>
         </is>
       </c>
     </row>
@@ -1202,19 +1202,19 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>76</v>
+        <v>194</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>59</v>
+        <v>160</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>74</v>
+        <v>195</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>31.3</v>
+        <v>26.7</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>32.43</v>
+        <v>55.9</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -1222,13 +1222,13 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>-57.8</v>
+        <v>7.8</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
@@ -1253,19 +1253,19 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>67</v>
+        <v>165</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>49</v>
+        <v>127</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>67</v>
+        <v>156</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>61</v>
+        <v>55.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>29.85</v>
+        <v>67.95</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -1273,13 +1273,13 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>-58.9</v>
+        <v>1.2</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
@@ -1300,23 +1300,23 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>智能视频分析</t>
+          <t>智慧农业感知</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>52</v>
+        <v>131</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>29</v>
+        <v>119</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>37</v>
+        <v>137</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>40.8</v>
+        <v>20.2</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>29.73</v>
+        <v>35.04</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -1324,13 +1324,13 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>-26.8</v>
+        <v>31</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
@@ -1351,23 +1351,23 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>智慧农业感知</t>
+          <t>智能视频分析</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>44</v>
+        <v>115</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.4</v>
+        <v>46.6</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>37.21</v>
+        <v>60.22</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -1375,13 +1375,13 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>-56</v>
+        <v>62</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
@@ -1402,27 +1402,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>环境监测</t>
+          <t>智慧畜牧</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>32</v>
+        <v>92</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>37</v>
+        <v>96</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>29.1</v>
+        <v>17.5</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>37.84</v>
+        <v>55.21</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
@@ -1432,7 +1432,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>-40.7</v>
+        <v>7</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
@@ -1453,37 +1453,37 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>智慧畜牧</t>
+          <t>环境监测</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>19.1</v>
+        <v>35.3</v>
       </c>
       <c r="H7" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2" t="n">
         <v>50</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>-66.3</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
@@ -1504,23 +1504,23 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>校园安全管理</t>
+          <t>智能仓储管理</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>25.1</v>
+        <v>28.7</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>36.36</v>
+        <v>55.71</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1528,13 +1528,13 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>-36.6</v>
+        <v>13.2</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
@@ -1555,37 +1555,37 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>室内外定位</t>
+          <t>楼宇能源管理</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>41.9</v>
+        <v>33.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>32</v>
+        <v>47.37</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>-57.1</v>
+        <v>70.5</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
@@ -1606,23 +1606,23 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>楼宇能源管理</t>
+          <t>校园安全管理</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>15.8</v>
+        <v>46.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>41.67</v>
+        <v>53.06</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1630,13 +1630,13 @@
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>-47.7</v>
+        <v>34.1</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -1661,19 +1661,19 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>75.2</v>
+        <v>42.2</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>36.84</v>
+        <v>72.22</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
@@ -1681,13 +1681,13 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
@@ -1708,37 +1708,37 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>智能仓储管理</t>
+          <t>室内外定位</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>36</v>
+        <v>42.2</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>30</v>
+        <v>65.91</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>-76.5</v>
+        <v>-19.6</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
@@ -1763,19 +1763,19 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>31.4</v>
+        <v>42.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>33.33</v>
+        <v>51.85</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -1789,7 +1789,7 @@
         <v>0</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>-50</v>
+        <v>22.7</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
@@ -11048,19 +11048,19 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>76</v>
+        <v>194</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>74</v>
+        <v>195</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>3.95</v>
+        <v>7.22</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0</v>
@@ -11088,19 +11088,19 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>67</v>
+        <v>165</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>67</v>
+        <v>156</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>13.43</v>
+        <v>10.91</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>0</v>
@@ -11124,23 +11124,23 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>智能视频分析</t>
+          <t>智慧农业感知</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>52</v>
+        <v>131</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>37</v>
+        <v>137</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>7.69</v>
+        <v>7.63</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>0</v>
@@ -11164,23 +11164,23 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>智慧农业感知</t>
+          <t>智能视频分析</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>44</v>
+        <v>115</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>13.64</v>
+        <v>11.3</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>0</v>
@@ -11204,14 +11204,14 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>环境监测</t>
+          <t>智慧畜牧</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>32</v>
+        <v>92</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>37</v>
+        <v>96</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>1</v>
@@ -11220,7 +11220,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>3.12</v>
+        <v>1.09</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>0</v>
@@ -11244,23 +11244,23 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>智慧畜牧</t>
+          <t>环境监测</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0</v>
+        <v>2.47</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>0</v>
@@ -11284,23 +11284,23 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>校园安全管理</t>
+          <t>智能仓储管理</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0</v>
+        <v>18.18</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0</v>
@@ -11324,23 +11324,23 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>室内外定位</t>
+          <t>楼宇能源管理</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>12.5</v>
+        <v>13.33</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0</v>
@@ -11364,23 +11364,23 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>楼宇能源管理</t>
+          <t>校园安全管理</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>8.699999999999999</v>
+        <v>5.45</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>0</v>
@@ -11408,19 +11408,19 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>41.18</v>
+        <v>21.57</v>
       </c>
       <c r="I11" s="2" t="n">
         <v>0</v>
@@ -11444,23 +11444,23 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>智能仓储管理</t>
+          <t>室内外定位</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>18.75</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="I12" s="2" t="n">
         <v>0</v>
@@ -11488,10 +11488,10 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>0</v>

</xml_diff>